<commit_message>
feat: synchronize spreadsheet structure and identity refs
</commit_message>
<xml_diff>
--- a/exemplos/controle_pipeline_flow.modelo.xlsx
+++ b/exemplos/controle_pipeline_flow.modelo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controle" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guia" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referencias_Identidade" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exemplo_Producao" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Controle" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Guia" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Referencias_Identidade" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Exemplo_Producao" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Controle'!$A$1:$AE$500</definedName>
@@ -828,7 +828,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>abertura, principal ou cta.</t>
+          <t>automatico, abertura, principal ou cta.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -843,7 +843,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Papel visual do arquivo principal.</t>
+          <t>base_edicao, produto, inspiracao, detalhe, ambiente, outro ou vazio.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -972,7 +972,7 @@
       <formula1>"sim,não"</formula1>
     </dataValidation>
     <dataValidation sqref="F4:F500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" promptTitle="Pipeline Flow" prompt="Escolha uma opção ou deixe vazio quando permitido." type="list">
-      <formula1>"abertura,principal,cta"</formula1>
+      <formula1>"automatico,abertura,principal,cta"</formula1>
     </dataValidation>
     <dataValidation sqref="I4:I500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" promptTitle="Pipeline Flow" prompt="Escolha uma opção ou deixe vazio quando permitido." type="list">
       <formula1>"base_edicao,produto,inspiração,detalhe,ambiente,outro"</formula1>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>abertura, principal ou cta.</t>
+          <t>automatico, abertura, principal ou cta.</t>
         </is>
       </c>
     </row>
@@ -1177,7 +1177,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Papel visual do arquivo principal.</t>
+          <t>base_edicao, produto, inspiracao, detalhe, ambiente, outro ou vazio.</t>
         </is>
       </c>
     </row>
@@ -1582,7 +1582,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>arquivo fictício</t>
+          <t>arquivo</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">

</xml_diff>